<commit_message>
FET: corrections in QMG-CFB Results
</commit_message>
<xml_diff>
--- a/earlyMBNMA-Forest_Plots/Time-course Adjusted Results - Overall/Table_05_QMG_score_improvement_from_baseline.xlsx
+++ b/earlyMBNMA-Forest_Plots/Time-course Adjusted Results - Overall/Table_05_QMG_score_improvement_from_baseline.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ebmhealth-my.sharepoint.com/personal/ananda_biswas_ebmhealth_in/Documents/Documents/R-Programs/earlyMBNMA-Forest_Plots/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ebmhealth-my.sharepoint.com/personal/ananda_biswas_ebmhealth_in/Documents/Documents/R-Programs/earlyMBNMA-Forest_Plots/Time-course Adjusted Results - Overall/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93E2C362-3976-4DC1-85E1-1BE9DCCB8D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{93E2C362-3976-4DC1-85E1-1BE9DCCB8D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BE7495E-3B1F-4AFF-A018-E1ADADC3F6E7}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6A840B43-5912-4ADB-AAEC-55F2674B12BF}"/>
   </bookViews>
@@ -34,15 +34,6 @@
     <t>upper</t>
   </si>
   <si>
-    <t>RTX 375mg</t>
-  </si>
-  <si>
-    <t>RAVU</t>
-  </si>
-  <si>
-    <t>SATR</t>
-  </si>
-  <si>
     <t>Rozanolixizumab_10mg</t>
   </si>
   <si>
@@ -86,6 +77,15 @@
   </si>
   <si>
     <t>Placebo</t>
+  </si>
+  <si>
+    <t>Rituximab_500mg</t>
+  </si>
+  <si>
+    <t>Ravulizumab</t>
+  </si>
+  <si>
+    <t>Satralizumab</t>
   </si>
 </sst>
 </file>
@@ -968,7 +968,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>-2.2799999999999998</v>
@@ -982,7 +982,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>-1.92</v>
@@ -996,7 +996,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>-1.66</v>
@@ -1010,7 +1010,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>-1.38</v>
@@ -1024,7 +1024,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B6">
         <v>-1.35</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>-1.1599999999999999</v>
@@ -1052,7 +1052,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B8">
         <v>-1.1499999999999999</v>
@@ -1066,7 +1066,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B9">
         <v>-1.07</v>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>-1</v>
@@ -1094,7 +1094,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>-0.95</v>
@@ -1108,7 +1108,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>-0.92</v>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>-0.62</v>
@@ -1136,7 +1136,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>-0.6</v>
@@ -1150,7 +1150,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B15">
         <v>-0.6</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B16">
         <v>-0.51</v>
@@ -1192,7 +1192,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <v>-0.32</v>
@@ -1206,7 +1206,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>0</v>

</xml_diff>